<commit_message>
Updated dealers again so it only has the newest dealer list.
</commit_message>
<xml_diff>
--- a/Wavcor Summary Leads.xlsx
+++ b/Wavcor Summary Leads.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wavcor.sharepoint.com/sites/WavcorInternational/Engineering/Software/Lead Tools/wix-odoo-webhook/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{19F13B64-00E5-F449-BA24-760B94091F98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{19F13B64-00E5-F449-BA24-760B94091F98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2B6F5037-3E1E-2F42-B1C7-861563425F79}"/>
   <bookViews>
-    <workbookView xWindow="160" yWindow="620" windowWidth="35940" windowHeight="19900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20920" yWindow="22320" windowWidth="35840" windowHeight="19900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="86" r:id="rId1"/>
@@ -11469,6 +11469,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="53" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="26.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="57">
@@ -43855,15 +43856,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="70a4a365-2753-4199-abdb-eb8db1d4debc" xsi:nil="true"/>
@@ -43874,7 +43866,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101001DBCBF14208C5B4D9DCB8B0E4F0A424D" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="665055633ffa4ea1ceac9e0b1b8aff7b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d5900feb-dde0-410c-80b8-c2962e8eda82" xmlns:ns3="70a4a365-2753-4199-abdb-eb8db1d4debc" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff70244a2ec93a669e69735a2af1e1ac" ns2:_="" ns3:_="">
     <xsd:import namespace="d5900feb-dde0-410c-80b8-c2962e8eda82"/>
@@ -44075,32 +44067,33 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{306E654B-0A5B-4952-9899-8BE4291BD587}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6E6D350-6E25-477B-B5DC-469D63AF66EF}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="d5900feb-dde0-410c-80b8-c2962e8eda82"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="70a4a365-2753-4199-abdb-eb8db1d4debc"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6E6D350-6E25-477B-B5DC-469D63AF66EF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="d5900feb-dde0-410c-80b8-c2962e8eda82"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="70a4a365-2753-4199-abdb-eb8db1d4debc"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4E902C50-8F83-4A3A-9ADC-CE38A8CCE144}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -44117,4 +44110,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{306E654B-0A5B-4952-9899-8BE4291BD587}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>